<commit_message>
Wrote the report map, wrote an untested press function and release function
</commit_message>
<xml_diff>
--- a/Research/HID Profile Specification.xlsx
+++ b/Research/HID Profile Specification.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cobingrosjean/Desktop/Mini_Macropad/Research/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC328323-1A73-DF47-AE44-C95DAA91B8B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{453842A9-F234-0649-B4FB-F52AACEDEE77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40960" yWindow="10180" windowWidth="34560" windowHeight="21680" xr2:uid="{E425E562-E31B-4E49-A568-3F33E203938C}"/>
+    <workbookView xWindow="40960" yWindow="10180" windowWidth="34560" windowHeight="21680" activeTab="1" xr2:uid="{E425E562-E31B-4E49-A568-3F33E203938C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="HID Over GATT Profile" sheetId="1" r:id="rId1"/>
+    <sheet name="Report Map Structure" sheetId="2" r:id="rId2"/>
+    <sheet name="Keyboard Report Structure" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="128">
   <si>
     <t>HID Service</t>
   </si>
@@ -174,18 +176,277 @@
   </si>
   <si>
     <t>0x2A29</t>
+  </si>
+  <si>
+    <t>Byte 1</t>
+  </si>
+  <si>
+    <t>Byte 2</t>
+  </si>
+  <si>
+    <t>Byte 3</t>
+  </si>
+  <si>
+    <t>Byte 4</t>
+  </si>
+  <si>
+    <t>Byte 5</t>
+  </si>
+  <si>
+    <t>Byte 6</t>
+  </si>
+  <si>
+    <t>Byte 7</t>
+  </si>
+  <si>
+    <t>Byte 0</t>
+  </si>
+  <si>
+    <t>Typical Implementation:</t>
+  </si>
+  <si>
+    <t>Modifier byte</t>
+  </si>
+  <si>
+    <t>Reserved byte</t>
+  </si>
+  <si>
+    <t>Keycode 2</t>
+  </si>
+  <si>
+    <t>Keycode 3</t>
+  </si>
+  <si>
+    <t>Keycode 1</t>
+  </si>
+  <si>
+    <t>Keycode 4</t>
+  </si>
+  <si>
+    <t>Keycode 5</t>
+  </si>
+  <si>
+    <t>Keycode 6</t>
+  </si>
+  <si>
+    <t>Whoever wrote these documents wrote them so poorly, and included so few examples, that it's a miracle that HID devices work at all</t>
+  </si>
+  <si>
+    <t>0x05</t>
+  </si>
+  <si>
+    <t>0x01</t>
+  </si>
+  <si>
+    <t>Usage Page</t>
+  </si>
+  <si>
+    <t>General Desktop Page</t>
+  </si>
+  <si>
+    <t>Item tag</t>
+  </si>
+  <si>
+    <t>Item value</t>
+  </si>
+  <si>
+    <t>Tag byte</t>
+  </si>
+  <si>
+    <t>Value byte</t>
+  </si>
+  <si>
+    <t>Usage</t>
+  </si>
+  <si>
+    <t>Keyboard</t>
+  </si>
+  <si>
+    <t>0x09</t>
+  </si>
+  <si>
+    <t>0x06</t>
+  </si>
+  <si>
+    <t>Logical Minimum</t>
+  </si>
+  <si>
+    <t>Logical Maximum</t>
+  </si>
+  <si>
+    <t>Report Size</t>
+  </si>
+  <si>
+    <t>Report Count</t>
+  </si>
+  <si>
+    <t>Collection</t>
+  </si>
+  <si>
+    <t>Application</t>
+  </si>
+  <si>
+    <t>0xA1</t>
+  </si>
+  <si>
+    <t>0x00</t>
+  </si>
+  <si>
+    <t>Item type</t>
+  </si>
+  <si>
+    <t>Main</t>
+  </si>
+  <si>
+    <t>Global</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>Keyboard/Keypad Page</t>
+  </si>
+  <si>
+    <t>0x07</t>
+  </si>
+  <si>
+    <t>Left Control</t>
+  </si>
+  <si>
+    <t>0x19</t>
+  </si>
+  <si>
+    <t>0xE0</t>
+  </si>
+  <si>
+    <t>Right GUI</t>
+  </si>
+  <si>
+    <t>0x29</t>
+  </si>
+  <si>
+    <t>0xE7</t>
+  </si>
+  <si>
+    <t>Usage Minimum</t>
+  </si>
+  <si>
+    <t>Usage Maximum</t>
+  </si>
+  <si>
+    <t>0x15</t>
+  </si>
+  <si>
+    <t>Zero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logical Maximum </t>
+  </si>
+  <si>
+    <t>One</t>
+  </si>
+  <si>
+    <t>0x25</t>
+  </si>
+  <si>
+    <t>0x75</t>
+  </si>
+  <si>
+    <t>Eight</t>
+  </si>
+  <si>
+    <t>0x95</t>
+  </si>
+  <si>
+    <t>0x08</t>
+  </si>
+  <si>
+    <t>Key Input</t>
+  </si>
+  <si>
+    <t>0x81</t>
+  </si>
+  <si>
+    <t>0x02</t>
+  </si>
+  <si>
+    <t>Data, Variable, Absolute</t>
+  </si>
+  <si>
+    <t>Reserved Byte</t>
+  </si>
+  <si>
+    <t>Constant (Useless Junk)</t>
+  </si>
+  <si>
+    <t>Constant</t>
+  </si>
+  <si>
+    <t>Keycode Array</t>
+  </si>
+  <si>
+    <t>0xFF</t>
+  </si>
+  <si>
+    <t>Data, array, absolute</t>
+  </si>
+  <si>
+    <t>End Collection</t>
+  </si>
+  <si>
+    <t>Doesn't matter</t>
+  </si>
+  <si>
+    <t>0xC0</t>
+  </si>
+  <si>
+    <t>Keyboard Report:</t>
+  </si>
+  <si>
+    <t>Report ID</t>
+  </si>
+  <si>
+    <t>0x85</t>
+  </si>
+  <si>
+    <t>Key Report</t>
+  </si>
+  <si>
+    <t>Consumer</t>
+  </si>
+  <si>
+    <t>0x0C</t>
+  </si>
+  <si>
+    <t>Consumer Control</t>
+  </si>
+  <si>
+    <t>Consumer Control Report (UNFINISHED)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -197,7 +458,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -205,12 +466,103 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -785,4 +1137,715 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F898F26-4B21-A249-8307-5141B6B5FD85}">
+  <dimension ref="A1:E64"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.5" customWidth="1"/>
+    <col min="2" max="2" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="10.5" customWidth="1"/>
+    <col min="6" max="6" width="9.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="5"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="6"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="8"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="8"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="6"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="8"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="C12" s="7">
+        <v>1</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="6"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="8"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="8"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="6"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="8"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="6"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="8"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="8"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="6"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="8"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" s="6"/>
+      <c r="B30" s="7"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="8"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B31" s="7"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="8"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" s="6"/>
+      <c r="B32" s="7"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="7"/>
+      <c r="E32" s="8"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="C34" s="7">
+        <v>0</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C35" s="7">
+        <v>255</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C36" s="7">
+        <v>0</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C37" s="7">
+        <v>1</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C38" s="7">
+        <v>8</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C39" s="7">
+        <v>6</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E40" s="11" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>86</v>
+      </c>
+      <c r="B46" t="s">
+        <v>121</v>
+      </c>
+      <c r="C46">
+        <v>2</v>
+      </c>
+      <c r="D46" t="s">
+        <v>122</v>
+      </c>
+      <c r="E46" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>86</v>
+      </c>
+      <c r="B50" t="s">
+        <v>66</v>
+      </c>
+      <c r="C50" t="s">
+        <v>124</v>
+      </c>
+      <c r="D50" t="s">
+        <v>64</v>
+      </c>
+      <c r="E50" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>87</v>
+      </c>
+      <c r="B51" t="s">
+        <v>72</v>
+      </c>
+      <c r="C51" t="s">
+        <v>126</v>
+      </c>
+      <c r="D51" t="s">
+        <v>74</v>
+      </c>
+      <c r="E51" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>86</v>
+      </c>
+      <c r="B52" t="s">
+        <v>76</v>
+      </c>
+      <c r="C52">
+        <v>0</v>
+      </c>
+      <c r="D52" t="s">
+        <v>98</v>
+      </c>
+      <c r="E52" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>86</v>
+      </c>
+      <c r="B53" t="s">
+        <v>77</v>
+      </c>
+      <c r="C53">
+        <v>1023</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>85</v>
+      </c>
+      <c r="B64" t="s">
+        <v>117</v>
+      </c>
+      <c r="C64" t="s">
+        <v>118</v>
+      </c>
+      <c r="D64" t="s">
+        <v>119</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{752FA69B-9688-1A45-97FE-1061EF053EC5}">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" t="s">
+        <v>58</v>
+      </c>
+      <c r="G2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H2" t="s">
+        <v>61</v>
+      </c>
+      <c r="I2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>